<commit_message>
Update type district model
</commit_message>
<xml_diff>
--- a/districtgenerator/data/typdistrict_parameters.xlsx
+++ b/districtgenerator/data/typdistrict_parameters.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PycharmProjects\districtgenerator\districtgenerator\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98343BDE-F620-4585-B04B-CD197FBBDE2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF6AA371-90C8-4927-8CC3-2FE29E0DE4B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{429C7893-B2AC-4DD2-A71C-1586DF0B06AF}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="89">
   <si>
     <t>Siedlungstyp</t>
   </si>
@@ -196,9 +196,6 @@
   </si>
   <si>
     <t>Ein- und Zweifamilienhaussiedlung niedriger Dichte</t>
-  </si>
-  <si>
-    <t>Einfamilienhaussiedlung hoher Dichte und Dorfkern</t>
   </si>
   <si>
     <t>Reihenhausbebauung</t>
@@ -299,6 +296,22 @@
   </si>
   <si>
     <t>Anzahl Vollgeschosse 100%</t>
+  </si>
+  <si>
+    <t>Nichtwohnnutzung (%)</t>
+  </si>
+  <si>
+    <t>Mischnutzung (%)</t>
+  </si>
+  <si>
+    <t>Wohnnutzung (%)</t>
+  </si>
+  <si>
+    <t>Siedlungsentwicklung und Infrastrukturfolgekosten - Bilanzierung und Strategieentwicklung
+https://www.ireus.uni-stuttgart.de/forschung/publikationen/Siedentop_etal_2006.pdf</t>
+  </si>
+  <si>
+    <t>Bausiedlung hoher Dichte und Dorfkern</t>
   </si>
 </sst>
 </file>
@@ -490,7 +503,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -539,6 +552,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -548,17 +573,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -874,7 +890,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36D4573D-B4BA-4F69-B051-517EE9D7E855}">
-  <dimension ref="A1:BD11"/>
+  <dimension ref="A1:BG11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="24.6640625" customWidth="1"/>
@@ -899,7 +915,7 @@
     <col min="56" max="56" width="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:56" ht="72">
+    <row r="1" spans="1:59" ht="72">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -961,10 +977,10 @@
         <v>34</v>
       </c>
       <c r="V1" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="W1" s="4" t="s">
         <v>60</v>
-      </c>
-      <c r="W1" s="4" t="s">
-        <v>61</v>
       </c>
       <c r="X1" s="1" t="s">
         <v>1</v>
@@ -1011,62 +1027,71 @@
       <c r="AL1" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="AM1" s="3" t="s">
+      <c r="AM1" s="20" t="s">
+        <v>84</v>
+      </c>
+      <c r="AN1" s="20" t="s">
+        <v>85</v>
+      </c>
+      <c r="AO1" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="AP1" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="AQ1" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="AN1" s="7" t="s">
+      <c r="AR1" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="AO1" s="7" t="s">
+      <c r="AS1" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="AP1" s="7" t="s">
+      <c r="AT1" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="AQ1" s="7" t="s">
+      <c r="AU1" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="AR1" s="7" t="s">
+      <c r="AV1" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="AS1" s="7" t="s">
+      <c r="AW1" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="AT1" s="7" t="s">
+      <c r="AX1" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="AU1" s="7" t="s">
+      <c r="AY1" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="AV1" s="4" t="s">
+      <c r="AZ1" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="AW1" s="3" t="s">
+      <c r="BA1" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="AX1" s="7" t="s">
+      <c r="BB1" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="AY1" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="AZ1" s="3" t="s">
+      <c r="BC1" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="BD1" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="BA1" s="7" t="s">
+      <c r="BE1" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="BB1" s="7" t="s">
+      <c r="BF1" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="BC1" s="7" t="s">
+      <c r="BG1" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="BD1" s="4" t="s">
-        <v>84</v>
-      </c>
     </row>
-    <row r="2" spans="1:56" ht="28.8">
+    <row r="2" spans="1:59" ht="28.8">
       <c r="A2" t="s">
         <v>44</v>
       </c>
@@ -1183,62 +1208,74 @@
       <c r="AL2" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="AM2" s="8">
-        <v>0</v>
+      <c r="AM2">
+        <f>20/(20+5+55)*100</f>
+        <v>25</v>
       </c>
       <c r="AN2">
+        <f>5/(20+5+55)*100</f>
+        <v>6.25</v>
+      </c>
+      <c r="AO2">
+        <f>55/(20+5+55)*100</f>
+        <v>68.75</v>
+      </c>
+      <c r="AP2" s="8">
+        <v>0</v>
+      </c>
+      <c r="AQ2">
         <v>37.5</v>
       </c>
-      <c r="AO2">
+      <c r="AR2">
         <v>42.5</v>
       </c>
-      <c r="AP2">
+      <c r="AS2">
         <v>17.5</v>
       </c>
-      <c r="AQ2">
+      <c r="AT2">
         <v>2.5</v>
       </c>
-      <c r="AR2">
-        <v>0</v>
-      </c>
-      <c r="AS2">
-        <v>0</v>
-      </c>
-      <c r="AT2">
-        <v>0</v>
-      </c>
       <c r="AU2">
         <v>0</v>
       </c>
-      <c r="AV2" s="9">
-        <v>0</v>
-      </c>
-      <c r="AW2" s="8">
+      <c r="AV2">
+        <v>0</v>
+      </c>
+      <c r="AW2">
+        <v>0</v>
+      </c>
+      <c r="AX2">
+        <v>0</v>
+      </c>
+      <c r="AY2" s="9">
+        <v>0</v>
+      </c>
+      <c r="AZ2" s="8">
         <v>35.9</v>
       </c>
-      <c r="AX2">
+      <c r="BA2">
         <v>51.4</v>
       </c>
-      <c r="AY2">
+      <c r="BB2">
         <v>4.3</v>
       </c>
-      <c r="AZ2" s="18">
+      <c r="BC2" s="18">
         <v>1</v>
       </c>
-      <c r="BA2">
+      <c r="BD2">
         <v>1</v>
       </c>
-      <c r="BB2">
+      <c r="BE2">
         <v>1.5</v>
       </c>
-      <c r="BC2">
+      <c r="BF2">
         <v>1.5</v>
       </c>
-      <c r="BD2" s="9">
+      <c r="BG2" s="9">
         <v>2.5</v>
       </c>
     </row>
-    <row r="3" spans="1:56" ht="28.8">
+    <row r="3" spans="1:59" ht="28.8">
       <c r="A3" t="s">
         <v>46</v>
       </c>
@@ -1355,62 +1392,74 @@
       <c r="AL3" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="AM3" s="8">
-        <v>0</v>
+      <c r="AM3">
+        <f>45/(45+10+25)*100</f>
+        <v>56.25</v>
       </c>
       <c r="AN3">
-        <v>0</v>
+        <f>10/(45+10+25)*100</f>
+        <v>12.5</v>
       </c>
       <c r="AO3">
+        <f>25/(45+10+25)*100</f>
+        <v>31.25</v>
+      </c>
+      <c r="AP3" s="8">
+        <v>0</v>
+      </c>
+      <c r="AQ3">
+        <v>0</v>
+      </c>
+      <c r="AR3">
         <v>8.6999999999999993</v>
       </c>
-      <c r="AP3">
+      <c r="AS3">
         <v>21.3</v>
       </c>
-      <c r="AQ3">
+      <c r="AT3">
         <v>24.7</v>
       </c>
-      <c r="AR3">
+      <c r="AU3">
         <v>16.7</v>
       </c>
-      <c r="AS3">
+      <c r="AV3">
         <v>17.3</v>
       </c>
-      <c r="AT3">
+      <c r="AW3">
         <v>8</v>
       </c>
-      <c r="AU3">
+      <c r="AX3">
         <v>3.3</v>
       </c>
-      <c r="AV3" s="9">
-        <v>0</v>
-      </c>
-      <c r="AW3" s="8">
+      <c r="AY3" s="9">
+        <v>0</v>
+      </c>
+      <c r="AZ3" s="8">
         <v>35.9</v>
       </c>
-      <c r="AX3">
+      <c r="BA3">
         <v>51.4</v>
       </c>
-      <c r="AY3">
+      <c r="BB3">
         <v>4.3</v>
       </c>
-      <c r="AZ3" s="18">
+      <c r="BC3" s="18">
         <v>1</v>
       </c>
-      <c r="BA3">
+      <c r="BD3">
         <v>1.5</v>
       </c>
-      <c r="BB3">
+      <c r="BE3">
         <v>2</v>
       </c>
-      <c r="BC3">
+      <c r="BF3">
         <v>2</v>
       </c>
-      <c r="BD3" s="9">
+      <c r="BG3" s="9">
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:56" ht="57.6">
+    <row r="4" spans="1:59" ht="57.6">
       <c r="A4" t="s">
         <v>45</v>
       </c>
@@ -1528,67 +1577,79 @@
       <c r="AL4" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="AM4" s="8">
+      <c r="AM4">
+        <f t="shared" ref="AM4:AN6" si="2">5/(5+5+70)*100</f>
+        <v>6.25</v>
+      </c>
+      <c r="AN4">
+        <f t="shared" si="2"/>
+        <v>6.25</v>
+      </c>
+      <c r="AO4">
+        <f>70/(5+5+70)*100</f>
+        <v>87.5</v>
+      </c>
+      <c r="AP4" s="8">
         <v>16.8</v>
       </c>
-      <c r="AN4">
+      <c r="AQ4">
         <v>14.5</v>
       </c>
-      <c r="AO4">
+      <c r="AR4">
         <v>9.9</v>
       </c>
-      <c r="AP4">
+      <c r="AS4">
         <v>10.7</v>
       </c>
-      <c r="AQ4">
+      <c r="AT4">
         <v>12.2</v>
       </c>
-      <c r="AR4">
+      <c r="AU4">
         <v>10.7</v>
       </c>
-      <c r="AS4">
+      <c r="AV4">
         <v>14.5</v>
       </c>
-      <c r="AT4">
+      <c r="AW4">
         <v>7.6</v>
       </c>
-      <c r="AU4">
+      <c r="AX4">
         <v>3.1</v>
       </c>
-      <c r="AV4" s="9">
-        <v>0</v>
-      </c>
-      <c r="AW4" s="8">
+      <c r="AY4" s="9">
+        <v>0</v>
+      </c>
+      <c r="AZ4" s="8">
         <v>35.9</v>
       </c>
-      <c r="AX4">
+      <c r="BA4">
         <v>51.4</v>
       </c>
-      <c r="AY4">
+      <c r="BB4">
         <v>4.3</v>
       </c>
-      <c r="AZ4" s="18">
+      <c r="BC4" s="18">
         <v>1</v>
       </c>
-      <c r="BA4">
+      <c r="BD4">
         <v>1</v>
       </c>
-      <c r="BB4">
+      <c r="BE4">
         <v>1.5</v>
       </c>
-      <c r="BC4">
+      <c r="BF4">
         <v>1.5</v>
       </c>
-      <c r="BD4" s="9">
+      <c r="BG4" s="9">
         <v>2.5</v>
       </c>
     </row>
-    <row r="5" spans="1:56" ht="28.8">
+    <row r="5" spans="1:59" ht="28.8">
       <c r="A5" t="s">
         <v>47</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>54</v>
+        <v>88</v>
       </c>
       <c r="C5" s="5">
         <v>0.2</v>
@@ -1625,7 +1686,7 @@
         <v>75</v>
       </c>
       <c r="N5" s="6">
-        <f t="shared" ref="N5:N7" si="2">L5*2-M5</f>
+        <f t="shared" ref="N5:N7" si="3">L5*2-M5</f>
         <v>155</v>
       </c>
       <c r="O5" s="5">
@@ -1701,67 +1762,79 @@
       <c r="AL5" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="AM5" s="8">
-        <v>0</v>
+      <c r="AM5">
+        <f t="shared" si="2"/>
+        <v>6.25</v>
       </c>
       <c r="AN5">
-        <v>0</v>
+        <f t="shared" si="2"/>
+        <v>6.25</v>
       </c>
       <c r="AO5">
+        <f>70/(5+5+70)*100</f>
+        <v>87.5</v>
+      </c>
+      <c r="AP5" s="8">
+        <v>0</v>
+      </c>
+      <c r="AQ5">
+        <v>0</v>
+      </c>
+      <c r="AR5">
         <v>8.6999999999999993</v>
       </c>
-      <c r="AP5">
+      <c r="AS5">
         <v>21.3</v>
       </c>
-      <c r="AQ5">
+      <c r="AT5">
         <v>24.7</v>
       </c>
-      <c r="AR5">
+      <c r="AU5">
         <v>16.7</v>
       </c>
-      <c r="AS5">
+      <c r="AV5">
         <v>17.3</v>
       </c>
-      <c r="AT5">
+      <c r="AW5">
         <v>8</v>
       </c>
-      <c r="AU5">
+      <c r="AX5">
         <v>3.3</v>
       </c>
-      <c r="AV5" s="9">
-        <v>0</v>
-      </c>
-      <c r="AW5" s="8">
+      <c r="AY5" s="9">
+        <v>0</v>
+      </c>
+      <c r="AZ5" s="8">
         <v>35.9</v>
       </c>
-      <c r="AX5">
+      <c r="BA5">
         <v>51.4</v>
       </c>
-      <c r="AY5">
+      <c r="BB5">
         <v>4.3</v>
       </c>
-      <c r="AZ5" s="18">
+      <c r="BC5" s="18">
         <v>1</v>
       </c>
-      <c r="BA5">
+      <c r="BD5">
         <v>1.5</v>
       </c>
-      <c r="BB5">
+      <c r="BE5">
         <v>2</v>
       </c>
-      <c r="BC5">
+      <c r="BF5">
         <v>2</v>
       </c>
-      <c r="BD5" s="9">
+      <c r="BG5" s="9">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:56" ht="28.8">
+    <row r="6" spans="1:59" ht="28.8">
       <c r="A6" t="s">
         <v>48</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C6" s="5">
         <v>0.2</v>
@@ -1798,7 +1871,7 @@
         <v>100</v>
       </c>
       <c r="N6" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>260</v>
       </c>
       <c r="O6" s="5">
@@ -1874,67 +1947,79 @@
       <c r="AL6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="AM6" s="8">
-        <v>0</v>
+      <c r="AM6">
+        <f t="shared" si="2"/>
+        <v>6.25</v>
       </c>
       <c r="AN6">
-        <v>0</v>
+        <f t="shared" si="2"/>
+        <v>6.25</v>
       </c>
       <c r="AO6">
+        <f>70/(5+5+70)*100</f>
+        <v>87.5</v>
+      </c>
+      <c r="AP6" s="8">
+        <v>0</v>
+      </c>
+      <c r="AQ6">
+        <v>0</v>
+      </c>
+      <c r="AR6">
         <v>8.6999999999999993</v>
       </c>
-      <c r="AP6">
+      <c r="AS6">
         <v>21.3</v>
       </c>
-      <c r="AQ6">
+      <c r="AT6">
         <v>24.7</v>
       </c>
-      <c r="AR6">
+      <c r="AU6">
         <v>16.7</v>
       </c>
-      <c r="AS6">
+      <c r="AV6">
         <v>17.3</v>
       </c>
-      <c r="AT6">
+      <c r="AW6">
         <v>8</v>
       </c>
-      <c r="AU6">
+      <c r="AX6">
         <v>3.3</v>
       </c>
-      <c r="AV6" s="9">
-        <v>0</v>
-      </c>
-      <c r="AW6" s="8">
+      <c r="AY6" s="9">
+        <v>0</v>
+      </c>
+      <c r="AZ6" s="8">
         <v>35.9</v>
       </c>
-      <c r="AX6">
+      <c r="BA6">
         <v>51.4</v>
       </c>
-      <c r="AY6">
+      <c r="BB6">
         <v>4.3</v>
       </c>
-      <c r="AZ6" s="18">
+      <c r="BC6" s="18">
         <v>1</v>
       </c>
-      <c r="BA6">
+      <c r="BD6">
         <v>1.5</v>
       </c>
-      <c r="BB6">
+      <c r="BE6">
         <v>2</v>
       </c>
-      <c r="BC6">
+      <c r="BF6">
         <v>2</v>
       </c>
-      <c r="BD6" s="9">
+      <c r="BG6" s="9">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:56" ht="57.6">
+    <row r="7" spans="1:59" ht="57.6">
       <c r="A7" t="s">
         <v>49</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C7" s="5">
         <v>0.4</v>
@@ -1971,7 +2056,7 @@
         <v>130</v>
       </c>
       <c r="N7" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>290</v>
       </c>
       <c r="O7" s="5">
@@ -2032,7 +2117,7 @@
       <c r="AG7" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="AH7" t="s">
+      <c r="AH7" s="27" t="s">
         <v>13</v>
       </c>
       <c r="AI7" s="2" t="s">
@@ -2047,67 +2132,79 @@
       <c r="AL7" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="AM7" s="8">
+      <c r="AM7">
+        <f>15/(15+5+60)*100</f>
+        <v>18.75</v>
+      </c>
+      <c r="AN7">
+        <f>5/(15+5+60)*100</f>
+        <v>6.25</v>
+      </c>
+      <c r="AO7">
+        <f>60/(15+5+60)*100</f>
+        <v>75</v>
+      </c>
+      <c r="AP7" s="8">
         <v>7.7</v>
       </c>
-      <c r="AN7">
+      <c r="AQ7">
         <v>20.5</v>
       </c>
-      <c r="AO7">
+      <c r="AR7">
         <v>23.2</v>
       </c>
-      <c r="AP7">
+      <c r="AS7">
         <v>17.899999999999999</v>
-      </c>
-      <c r="AQ7">
-        <v>5.0999999999999996</v>
-      </c>
-      <c r="AR7">
-        <v>7.7</v>
-      </c>
-      <c r="AS7">
-        <v>7.7</v>
       </c>
       <c r="AT7">
         <v>5.0999999999999996</v>
       </c>
       <c r="AU7">
+        <v>7.7</v>
+      </c>
+      <c r="AV7">
+        <v>7.7</v>
+      </c>
+      <c r="AW7">
         <v>5.0999999999999996</v>
       </c>
-      <c r="AV7" s="9">
-        <v>0</v>
-      </c>
-      <c r="AW7" s="8">
+      <c r="AX7">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="AY7" s="9">
+        <v>0</v>
+      </c>
+      <c r="AZ7" s="8">
         <v>35.9</v>
       </c>
-      <c r="AX7">
+      <c r="BA7">
         <v>51.4</v>
       </c>
-      <c r="AY7">
+      <c r="BB7">
         <v>4.3</v>
       </c>
-      <c r="AZ7" s="18">
+      <c r="BC7" s="18">
         <v>4</v>
       </c>
-      <c r="BA7">
+      <c r="BD7">
         <v>4</v>
       </c>
-      <c r="BB7">
+      <c r="BE7">
         <v>4</v>
       </c>
-      <c r="BC7">
+      <c r="BF7">
         <v>4</v>
       </c>
-      <c r="BD7" s="9">
+      <c r="BG7" s="9">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:56" ht="28.8">
+    <row r="8" spans="1:59" ht="28.8">
       <c r="A8" t="s">
         <v>50</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C8" s="5">
         <v>0.8</v>
@@ -2219,67 +2316,79 @@
       <c r="AL8" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="AM8" s="8">
-        <v>0</v>
+      <c r="AM8">
+        <f>5/(5+5+70)*100</f>
+        <v>6.25</v>
       </c>
       <c r="AN8">
-        <v>0</v>
+        <f>5/(5+5+70)*100</f>
+        <v>6.25</v>
       </c>
       <c r="AO8">
-        <v>0</v>
-      </c>
-      <c r="AP8">
+        <f>70/(5+5+70)*100</f>
+        <v>87.5</v>
+      </c>
+      <c r="AP8" s="8">
         <v>0</v>
       </c>
       <c r="AQ8">
+        <v>0</v>
+      </c>
+      <c r="AR8">
+        <v>0</v>
+      </c>
+      <c r="AS8">
+        <v>0</v>
+      </c>
+      <c r="AT8">
         <v>44.5</v>
       </c>
-      <c r="AR8">
+      <c r="AU8">
         <v>22.2</v>
       </c>
-      <c r="AS8">
+      <c r="AV8">
         <v>11.1</v>
       </c>
-      <c r="AT8">
+      <c r="AW8">
         <v>11.1</v>
       </c>
-      <c r="AU8">
+      <c r="AX8">
         <v>11.1</v>
       </c>
-      <c r="AV8" s="9">
-        <v>0</v>
-      </c>
-      <c r="AW8" s="8">
+      <c r="AY8" s="9">
+        <v>0</v>
+      </c>
+      <c r="AZ8" s="8">
         <v>35.9</v>
       </c>
-      <c r="AX8">
+      <c r="BA8">
         <v>51.4</v>
       </c>
-      <c r="AY8">
+      <c r="BB8">
         <v>4.3</v>
       </c>
-      <c r="AZ8" s="18">
+      <c r="BC8" s="18">
         <v>6.5</v>
       </c>
-      <c r="BA8">
+      <c r="BD8">
         <v>7.5</v>
       </c>
-      <c r="BB8">
+      <c r="BE8">
         <v>9</v>
       </c>
-      <c r="BC8">
+      <c r="BF8">
         <v>11</v>
       </c>
-      <c r="BD8" s="9">
+      <c r="BG8" s="9">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:56" ht="28.8">
+    <row r="9" spans="1:59" ht="28.8">
       <c r="A9" t="s">
         <v>6</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C9" s="5">
         <v>0.5</v>
@@ -2392,21 +2501,24 @@
       <c r="AL9" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="AM9" s="8">
+      <c r="AM9">
+        <f>20/(20+15+45)*100</f>
+        <v>25</v>
+      </c>
+      <c r="AN9">
+        <f>15/(20+15+45)*100</f>
+        <v>18.75</v>
+      </c>
+      <c r="AO9">
+        <f>45/(20+15+45)*100</f>
+        <v>56.25</v>
+      </c>
+      <c r="AP9" s="8">
         <v>46.9</v>
       </c>
-      <c r="AN9">
+      <c r="AQ9">
         <v>53.1</v>
       </c>
-      <c r="AO9">
-        <v>0</v>
-      </c>
-      <c r="AP9">
-        <v>0</v>
-      </c>
-      <c r="AQ9">
-        <v>0</v>
-      </c>
       <c r="AR9">
         <v>0</v>
       </c>
@@ -2419,40 +2531,49 @@
       <c r="AU9">
         <v>0</v>
       </c>
-      <c r="AV9" s="9">
-        <v>0</v>
-      </c>
-      <c r="AW9" s="8">
+      <c r="AV9">
+        <v>0</v>
+      </c>
+      <c r="AW9">
+        <v>0</v>
+      </c>
+      <c r="AX9">
+        <v>0</v>
+      </c>
+      <c r="AY9" s="9">
+        <v>0</v>
+      </c>
+      <c r="AZ9" s="8">
         <v>35.9</v>
       </c>
-      <c r="AX9">
+      <c r="BA9">
         <v>51.4</v>
       </c>
-      <c r="AY9">
+      <c r="BB9">
         <v>4.3</v>
       </c>
-      <c r="AZ9" s="18">
+      <c r="BC9" s="18">
         <v>2</v>
       </c>
-      <c r="BA9">
+      <c r="BD9">
         <v>3</v>
       </c>
-      <c r="BB9">
+      <c r="BE9">
         <v>4</v>
       </c>
-      <c r="BC9">
+      <c r="BF9">
         <v>5</v>
       </c>
-      <c r="BD9" s="9">
+      <c r="BG9" s="9">
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:56" ht="29.4" thickBot="1">
+    <row r="10" spans="1:59" ht="29.4" thickBot="1">
       <c r="A10" t="s">
         <v>51</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C10" s="16">
         <v>1.5</v>
@@ -2565,21 +2686,24 @@
       <c r="AL10" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="AM10" s="10">
+      <c r="AM10">
+        <f>20/(20+15+45)*100</f>
+        <v>25</v>
+      </c>
+      <c r="AN10">
+        <f>15/(20+15+45)*100</f>
+        <v>18.75</v>
+      </c>
+      <c r="AO10">
+        <f>45/(20+15+45)*100</f>
+        <v>56.25</v>
+      </c>
+      <c r="AP10" s="10">
         <v>86.2</v>
       </c>
-      <c r="AN10" s="14">
+      <c r="AQ10" s="14">
         <v>13.8</v>
       </c>
-      <c r="AO10" s="14">
-        <v>0</v>
-      </c>
-      <c r="AP10" s="14">
-        <v>0</v>
-      </c>
-      <c r="AQ10" s="14">
-        <v>0</v>
-      </c>
       <c r="AR10" s="14">
         <v>0</v>
       </c>
@@ -2592,108 +2716,123 @@
       <c r="AU10" s="14">
         <v>0</v>
       </c>
-      <c r="AV10" s="11">
-        <v>0</v>
-      </c>
-      <c r="AW10" s="10">
+      <c r="AV10" s="14">
+        <v>0</v>
+      </c>
+      <c r="AW10" s="14">
+        <v>0</v>
+      </c>
+      <c r="AX10" s="14">
+        <v>0</v>
+      </c>
+      <c r="AY10" s="11">
+        <v>0</v>
+      </c>
+      <c r="AZ10" s="10">
         <v>35.9</v>
       </c>
-      <c r="AX10" s="14">
+      <c r="BA10" s="14">
         <v>51.4</v>
       </c>
-      <c r="AY10" s="14">
+      <c r="BB10" s="14">
         <v>4.3</v>
       </c>
-      <c r="AZ10" s="19">
+      <c r="BC10" s="19">
         <v>2.5</v>
       </c>
-      <c r="BA10" s="14">
+      <c r="BD10" s="14">
         <v>3.5</v>
       </c>
-      <c r="BB10" s="14">
+      <c r="BE10" s="14">
         <v>3.5</v>
       </c>
-      <c r="BC10" s="14">
+      <c r="BF10" s="14">
         <v>4.5</v>
       </c>
-      <c r="BD10" s="11">
+      <c r="BG10" s="11">
         <v>6.5</v>
       </c>
     </row>
-    <row r="11" spans="1:56" ht="105" customHeight="1" thickBot="1">
+    <row r="11" spans="1:59" ht="105" customHeight="1" thickBot="1">
       <c r="A11" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="B11" s="24" t="s">
         <v>75</v>
       </c>
-      <c r="B11" s="20" t="s">
+      <c r="C11" s="25"/>
+      <c r="D11" s="25"/>
+      <c r="E11" s="25"/>
+      <c r="F11" s="25"/>
+      <c r="G11" s="25"/>
+      <c r="H11" s="25"/>
+      <c r="I11" s="25"/>
+      <c r="J11" s="25"/>
+      <c r="K11" s="25"/>
+      <c r="L11" s="25"/>
+      <c r="M11" s="25"/>
+      <c r="N11" s="25"/>
+      <c r="O11" s="25"/>
+      <c r="P11" s="25"/>
+      <c r="Q11" s="25"/>
+      <c r="R11" s="25"/>
+      <c r="S11" s="25"/>
+      <c r="T11" s="25"/>
+      <c r="U11" s="25"/>
+      <c r="V11" s="25"/>
+      <c r="W11" s="25"/>
+      <c r="X11" s="25"/>
+      <c r="Y11" s="25"/>
+      <c r="Z11" s="25"/>
+      <c r="AA11" s="25"/>
+      <c r="AB11" s="25"/>
+      <c r="AC11" s="25"/>
+      <c r="AD11" s="25"/>
+      <c r="AE11" s="25"/>
+      <c r="AF11" s="25"/>
+      <c r="AG11" s="25"/>
+      <c r="AH11" s="25"/>
+      <c r="AI11" s="25"/>
+      <c r="AJ11" s="25"/>
+      <c r="AK11" s="25"/>
+      <c r="AL11" s="26"/>
+      <c r="AM11" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="AN11" s="22"/>
+      <c r="AO11" s="22"/>
+      <c r="AP11" s="21" t="s">
         <v>76</v>
       </c>
-      <c r="C11" s="21"/>
-      <c r="D11" s="21"/>
-      <c r="E11" s="21"/>
-      <c r="F11" s="21"/>
-      <c r="G11" s="21"/>
-      <c r="H11" s="21"/>
-      <c r="I11" s="21"/>
-      <c r="J11" s="21"/>
-      <c r="K11" s="21"/>
-      <c r="L11" s="21"/>
-      <c r="M11" s="21"/>
-      <c r="N11" s="21"/>
-      <c r="O11" s="21"/>
-      <c r="P11" s="21"/>
-      <c r="Q11" s="21"/>
-      <c r="R11" s="21"/>
-      <c r="S11" s="21"/>
-      <c r="T11" s="21"/>
-      <c r="U11" s="21"/>
-      <c r="V11" s="21"/>
-      <c r="W11" s="21"/>
-      <c r="X11" s="21"/>
-      <c r="Y11" s="21"/>
-      <c r="Z11" s="21"/>
-      <c r="AA11" s="21"/>
-      <c r="AB11" s="21"/>
-      <c r="AC11" s="21"/>
-      <c r="AD11" s="21"/>
-      <c r="AE11" s="21"/>
-      <c r="AF11" s="21"/>
-      <c r="AG11" s="21"/>
-      <c r="AH11" s="21"/>
-      <c r="AI11" s="21"/>
-      <c r="AJ11" s="21"/>
-      <c r="AK11" s="21"/>
-      <c r="AL11" s="22"/>
-      <c r="AM11" s="23" t="s">
+      <c r="AQ11" s="22"/>
+      <c r="AR11" s="22"/>
+      <c r="AS11" s="22"/>
+      <c r="AT11" s="22"/>
+      <c r="AU11" s="22"/>
+      <c r="AV11" s="22"/>
+      <c r="AW11" s="22"/>
+      <c r="AX11" s="22"/>
+      <c r="AY11" s="23"/>
+      <c r="AZ11" s="21" t="s">
         <v>77</v>
       </c>
-      <c r="AN11" s="21"/>
-      <c r="AO11" s="21"/>
-      <c r="AP11" s="21"/>
-      <c r="AQ11" s="21"/>
-      <c r="AR11" s="21"/>
-      <c r="AS11" s="21"/>
-      <c r="AT11" s="21"/>
-      <c r="AU11" s="21"/>
-      <c r="AV11" s="22"/>
-      <c r="AW11" s="23" t="s">
+      <c r="BA11" s="22"/>
+      <c r="BB11" s="23"/>
+      <c r="BC11" s="21" t="s">
         <v>78</v>
       </c>
-      <c r="AX11" s="21"/>
-      <c r="AY11" s="22"/>
-      <c r="AZ11" s="24" t="s">
-        <v>79</v>
-      </c>
-      <c r="BA11" s="25"/>
-      <c r="BB11" s="25"/>
-      <c r="BC11" s="25"/>
-      <c r="BD11" s="26"/>
+      <c r="BD11" s="22"/>
+      <c r="BE11" s="22"/>
+      <c r="BF11" s="22"/>
+      <c r="BG11" s="23"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
+    <mergeCell ref="AZ11:BB11"/>
+    <mergeCell ref="BC11:BG11"/>
+    <mergeCell ref="AM11:AO11"/>
     <mergeCell ref="B11:AL11"/>
-    <mergeCell ref="AM11:AV11"/>
-    <mergeCell ref="AW11:AY11"/>
-    <mergeCell ref="AZ11:BD11"/>
+    <mergeCell ref="AP11:AY11"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <conditionalFormatting sqref="C2:C10">

</xml_diff>